<commit_message>
Weekly ML Hires Signal — 2026-05-29
</commit_message>
<xml_diff>
--- a/output/ML_Hires_Signal_2026-05-29.xlsx
+++ b/output/ML_Hires_Signal_2026-05-29.xlsx
@@ -33,7 +33,7 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="00276221"/>
+      <color rgb="009C6500"/>
       <sz val="10"/>
     </font>
     <font>
@@ -55,7 +55,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -593,7 +593,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -606,52 +606,50 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Qualcomm Inc.</t>
+          <t>NVIDIA Corporation</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>qualcomm.com</t>
+          <t>nvidia.com</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G2" s="2" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +29 new ML roles WoW</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J2" s="3" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
+        <v>20</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>2026 Intern-Machine Learning &amp;Multimedia Software Engineer</t>
+          <t>Principal Deep Learning Communication Architect</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
@@ -660,7 +658,7 @@
         </is>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>38962</v>
+        <v>130497</v>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
@@ -676,7 +674,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -689,61 +687,59 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Tesla Inc.</t>
+          <t>Oracle Corporation</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>tesla.com</t>
+          <t>oracle.com</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +21 new ML roles WoW</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J3" s="3" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>Site Reliability Engineer, HPC / AI Infrastructure</t>
+          <t>[Remote] Principal Applied Scientist</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
         <is>
-          <t>EV / Auto</t>
+          <t>Software / Cloud</t>
         </is>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>97690</v>
+        <v>52961</v>
       </c>
       <c r="R3" s="3" t="inlineStr">
         <is>
@@ -759,7 +755,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -772,63 +768,59 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>NVIDIA Corporation</t>
+          <t>Microsoft Corporation</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>nvidia.com</t>
+          <t>microsoft.com</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +20 new ML roles WoW</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J4" s="3" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
+        <v>6</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>Principal Deep Learning Communication Architect</t>
+          <t>Principal Applied Scientist (CoreAI)</t>
         </is>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>130497</v>
+        <v>245122</v>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
@@ -844,7 +836,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -852,68 +844,62 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>POD 4 Banking Payments Insurance</t>
+          <t>POD 5 Consumer Internet Software Auto</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>JPMorgan Chase &amp; Co.</t>
+          <t>Uber Technologies</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>jpmorganchase.com</t>
+          <t>uber.com</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +19 new ML roles WoW</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J5" s="3" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
+        <v>7</v>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>Product Director Speech and Voice AI/ML</t>
+          <t>Senior Data Scientist - Applied AI</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
         <is>
-          <t>Money Center Bank</t>
+          <t>Mobility / Delivery</t>
         </is>
       </c>
       <c r="Q5" s="2" t="n">
-        <v>177421</v>
+        <v>43970</v>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
@@ -929,7 +915,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -942,54 +928,50 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Citigroup Inc.</t>
+          <t>JPMorgan Chase &amp; Co.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>citigroup.com</t>
+          <t>jpmorganchase.com</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G6" s="2" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +18 new ML roles WoW</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J6" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
+        <v>19</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M6" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>Lead AI Engineer, Banking Technology - Senior Vice President</t>
+          <t>Product Director Speech and Voice AI/ML</t>
         </is>
       </c>
       <c r="P6" s="3" t="inlineStr">
@@ -998,7 +980,7 @@
         </is>
       </c>
       <c r="Q6" s="2" t="n">
-        <v>71355</v>
+        <v>177421</v>
       </c>
       <c r="R6" s="3" t="inlineStr">
         <is>
@@ -1014,7 +996,7 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -1022,68 +1004,60 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>POD 4 Banking Payments Insurance</t>
+          <t>POD 6 Cyber Telco Retail M&amp;E</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Mastercard Incorporated</t>
+          <t>Target Corporation</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>mastercard.com</t>
+          <t>target.com</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +14 new ML roles WoW</t>
+          <t>Director+ hiring</t>
         </is>
       </c>
       <c r="J7" s="3" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>Principal AI Engineer</t>
+          <t>Principal AI Engineer-Advanced AI</t>
         </is>
       </c>
       <c r="P7" s="3" t="inlineStr">
         <is>
-          <t>Payment Networks</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="Q7" s="2" t="n">
-        <v>28167</v>
+        <v>107412</v>
       </c>
       <c r="R7" s="3" t="inlineStr">
         <is>
@@ -1099,7 +1073,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -1107,66 +1081,64 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>POD 5 Consumer Internet Software Auto</t>
+          <t>POD 2 Healthcare &amp; Life Sciences</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
+          <t>Pfizer Inc.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>apple.com</t>
+          <t>pfizer.com</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +13 new ML roles WoW</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J8" s="3" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer – Edge AI &amp; On-Device Optimization</t>
+          <t>Principal Statistical Data Scientist</t>
         </is>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Consumer Tech</t>
+          <t>Pharmaceuticals</t>
         </is>
       </c>
       <c r="Q8" s="2" t="n">
-        <v>391035</v>
+        <v>63627</v>
       </c>
       <c r="R8" s="3" t="inlineStr">
         <is>
@@ -1182,7 +1154,7 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -1205,33 +1177,29 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +8 new ML roles WoW</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J9" s="3" t="n">
         <v>8</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
@@ -1265,7 +1233,7 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -1273,68 +1241,62 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>POD 6 Cyber Telco Retail M&amp;E</t>
+          <t>POD 4 Banking Payments Insurance</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Walmart Inc.</t>
+          <t>PayPal Holdings</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>walmart.com</t>
+          <t>paypal.com</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +8 new ML roles WoW</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J10" s="3" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>(USA) Principal, Data Scientist - Applied AI</t>
+          <t>Sr Machine Learning Engineer — Agentic Systems</t>
         </is>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Payments</t>
         </is>
       </c>
       <c r="Q10" s="2" t="n">
-        <v>648125</v>
+        <v>31797</v>
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
@@ -1350,7 +1312,7 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
@@ -1363,43 +1325,39 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Netflix Inc.</t>
+          <t>Apple Inc.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>netflix.com</t>
+          <t>apple.com</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +8 new ML roles WoW</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J11" s="3" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
@@ -1408,16 +1366,16 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Data Scientist 5 - TV &amp; Interactive Discovery</t>
+          <t>Machine Learning Engineer – Edge AI &amp; On-Device Optimization</t>
         </is>
       </c>
       <c r="P11" s="3" t="inlineStr">
         <is>
-          <t>Streaming</t>
+          <t>Consumer Tech</t>
         </is>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>39001</v>
+        <v>391035</v>
       </c>
       <c r="R11" s="3" t="inlineStr">
         <is>
@@ -1433,7 +1391,7 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -1446,43 +1404,39 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Uber Technologies</t>
+          <t>Intel Corporation</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>uber.com</t>
+          <t>intel.com</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +7 new ML roles WoW</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J12" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
@@ -1491,16 +1445,16 @@
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Senior Data Scientist - Applied AI</t>
+          <t>Senior GenAI Software Solutions Engineer</t>
         </is>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>Mobility / Delivery</t>
+          <t>Semiconductors</t>
         </is>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>43970</v>
+        <v>53101</v>
       </c>
       <c r="R12" s="3" t="inlineStr">
         <is>
@@ -1516,7 +1470,7 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -1524,68 +1478,64 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>POD 5 Consumer Internet Software Auto</t>
+          <t>POD 6 Cyber Telco Retail M&amp;E</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Microsoft Corporation</t>
+          <t>Walmart Inc.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>microsoft.com</t>
+          <t>walmart.com</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G13" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +6 new ML roles WoW</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J13" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>Principal Applied Scientist (CoreAI)</t>
+          <t>(USA) Principal, Data Scientist - Applied AI</t>
         </is>
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>245122</v>
+        <v>648125</v>
       </c>
       <c r="R13" s="3" t="inlineStr">
         <is>
@@ -1601,7 +1551,7 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
@@ -1609,68 +1559,60 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>POD 5 Consumer Internet Software Auto</t>
+          <t>POD 1 Capital Markets</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Oracle Corporation</t>
+          <t>BlackRock Inc.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>oracle.com</t>
+          <t>blackrock.com</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G14" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +5 new ML roles WoW</t>
+          <t>Director+ hiring</t>
         </is>
       </c>
       <c r="J14" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="N14" s="2" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>[Remote] Principal Applied Scientist</t>
+          <t>Alpha Generation Applied AI Engineer, Vice President</t>
         </is>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>Software / Cloud</t>
+          <t>Asset Management</t>
         </is>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>52961</v>
+        <v>20407</v>
       </c>
       <c r="R14" s="3" t="inlineStr">
         <is>
@@ -1686,7 +1628,7 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
@@ -1694,66 +1636,58 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>POD 5 Consumer Internet Software Auto</t>
+          <t>POD 1 Capital Markets</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Salesforce Inc.</t>
+          <t>Intercontinental Exchange</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>salesforce.com</t>
+          <t>ice.com</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +5 new ML roles WoW</t>
+          <t>1 active ML roles</t>
         </is>
       </c>
       <c r="J15" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>Lead AI Engineer, Data Solutions</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="P15" s="3" t="inlineStr">
         <is>
-          <t>SaaS</t>
+          <t>Exchanges</t>
         </is>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>37895</v>
+        <v>9333</v>
       </c>
       <c r="R15" s="3" t="inlineStr">
         <is>
@@ -1769,7 +1703,7 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -1777,66 +1711,58 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>POD 5 Consumer Internet Software Auto</t>
+          <t>POD 2 Healthcare &amp; Life Sciences</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Intel Corporation</t>
+          <t>Abbott Laboratories</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>intel.com</t>
+          <t>abbott.com</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +4 ML roles added</t>
+          <t>1 active ML roles</t>
         </is>
       </c>
       <c r="J16" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>Senior GenAI Software Solutions Engineer</t>
+          <t>Senior Clinical Research Scientist</t>
         </is>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>Semiconductors</t>
+          <t>Medical Devices</t>
         </is>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>53101</v>
+        <v>41950</v>
       </c>
       <c r="R16" s="3" t="inlineStr">
         <is>
@@ -1852,7 +1778,7 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
@@ -1860,66 +1786,64 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>POD 6 Cyber Telco Retail M&amp;E</t>
+          <t>POD 2 Healthcare &amp; Life Sciences</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>T-Mobile US Inc.</t>
+          <t>AbbVie Inc.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>t-mobile.com</t>
+          <t>abbvie.com</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +4 ML roles added</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J17" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>T Hub - AI Intern – LLM, Voice to Text &amp; Agentic Systems</t>
+          <t>Principal Research Scientist II - Process Chemistry</t>
         </is>
       </c>
       <c r="P17" s="3" t="inlineStr">
         <is>
-          <t>Telco</t>
+          <t>Pharmaceuticals</t>
         </is>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>81400</v>
+        <v>56334</v>
       </c>
       <c r="R17" s="3" t="inlineStr">
         <is>
@@ -1935,7 +1859,7 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -1943,64 +1867,62 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>POD 6 Cyber Telco Retail M&amp;E</t>
+          <t>POD 2 Healthcare &amp; Life Sciences</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Target Corporation</t>
+          <t>Amgen Inc.</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>target.com</t>
+          <t>amgen.com</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; +3 ML roles added</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J18" s="3" t="n">
         <v>3</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>Principal AI Engineer-Advanced AI</t>
+          <t>Sr Machine Learning Engineer</t>
         </is>
       </c>
       <c r="P18" s="3" t="inlineStr">
         <is>
-          <t>Retail</t>
+          <t>Biotech</t>
         </is>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>107412</v>
+        <v>33424</v>
       </c>
       <c r="R18" s="3" t="inlineStr">
         <is>
@@ -2016,7 +1938,7 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
@@ -2029,63 +1951,53 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Pfizer Inc.</t>
+          <t>Humana Inc.</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>pfizer.com</t>
+          <t>humana.com</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +3 ML roles added</t>
+          <t>3 active ML roles</t>
         </is>
       </c>
       <c r="J19" s="3" t="n">
         <v>3</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Principal Statistical Data Scientist</t>
+          <t>Infrastructure Operations Lead Cloud and AI GenAI Enablement</t>
         </is>
       </c>
       <c r="P19" s="3" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
+          <t>Managed Care</t>
         </is>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>63627</v>
+        <v>117761</v>
       </c>
       <c r="R19" s="3" t="inlineStr">
         <is>
@@ -2101,7 +2013,7 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
@@ -2109,64 +2021,62 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>POD 1 Capital Markets</t>
+          <t>POD 3 Manufacturing &amp; Robotics</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>BlackRock Inc.</t>
+          <t>Boeing Company</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>blackrock.com</t>
+          <t>boeing.com</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; +3 ML roles added</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J20" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M20" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Alpha Generation Applied AI Engineer, Vice President</t>
+          <t>AI/ML Researcher (Multimodal)</t>
         </is>
       </c>
       <c r="P20" s="3" t="inlineStr">
         <is>
-          <t>Asset Management</t>
+          <t>Aerospace</t>
         </is>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>20407</v>
+        <v>77794</v>
       </c>
       <c r="R20" s="3" t="inlineStr">
         <is>
@@ -2182,7 +2092,7 @@
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
@@ -2190,48 +2100,44 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>POD 2 Healthcare &amp; Life Sciences</t>
+          <t>POD 3 Manufacturing &amp; Robotics</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>AbbVie Inc.</t>
+          <t>Honeywell International</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>abbvie.com</t>
+          <t>honeywell.com</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +3 ML roles added</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
       <c r="M21" s="2" t="n">
         <v>1</v>
       </c>
@@ -2242,16 +2148,16 @@
       </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>Principal Research Scientist II - Process Chemistry</t>
+          <t>Principal AI Engineer</t>
         </is>
       </c>
       <c r="P21" s="3" t="inlineStr">
         <is>
-          <t>Pharmaceuticals</t>
+          <t>Industrial Conglomerate</t>
         </is>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>56334</v>
+        <v>37847</v>
       </c>
       <c r="R21" s="3" t="inlineStr">
         <is>
@@ -2267,7 +2173,7 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -2275,48 +2181,44 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>POD 2 Healthcare &amp; Life Sciences</t>
+          <t>POD 3 Manufacturing &amp; Robotics</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Amgen Inc.</t>
+          <t>Jacobs Solutions Inc.</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>amgen.com</t>
+          <t>jacobs.com</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +3 ML roles added</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J22" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr"/>
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
@@ -2325,16 +2227,16 @@
       </c>
       <c r="O22" s="3" t="inlineStr">
         <is>
-          <t>Sr Machine Learning Engineer</t>
+          <t>Senior AI/Data Platform Engineer (Snowflake, GenAI)</t>
         </is>
       </c>
       <c r="P22" s="3" t="inlineStr">
         <is>
-          <t>Biotech</t>
+          <t>Engineering / Defense</t>
         </is>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>33424</v>
+        <v>16751</v>
       </c>
       <c r="R22" s="3" t="inlineStr">
         <is>
@@ -2350,7 +2252,7 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
@@ -2358,62 +2260,58 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>POD 2 Healthcare &amp; Life Sciences</t>
+          <t>POD 4 Banking Payments Insurance</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Humana Inc.</t>
+          <t>AIG (American Intl. Group)</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>humana.com</t>
+          <t>aig.com</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>+3 ML roles added</t>
+          <t>1 active ML roles</t>
         </is>
       </c>
       <c r="J23" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr"/>
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>Infrastructure Operations Lead Cloud and AI GenAI Enablement</t>
+          <t>Ph.D. Research Data Scientist, GenAI</t>
         </is>
       </c>
       <c r="P23" s="3" t="inlineStr">
         <is>
-          <t>Managed Care</t>
+          <t>P&amp;C Insurance</t>
         </is>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>117761</v>
+        <v>46951</v>
       </c>
       <c r="R23" s="3" t="inlineStr">
         <is>
@@ -2429,7 +2327,7 @@
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -2437,68 +2335,64 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>POD 3 Manufacturing &amp; Robotics</t>
+          <t>POD 4 Banking Payments Insurance</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Honeywell International</t>
+          <t>Citigroup Inc.</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>honeywell.com</t>
+          <t>citigroup.com</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +3 ML roles added</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J24" s="3" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
+        <v>18</v>
+      </c>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>Principal AI Engineer</t>
+          <t>Lead AI Engineer, Banking Technology - Senior Vice President</t>
         </is>
       </c>
       <c r="P24" s="3" t="inlineStr">
         <is>
-          <t>Industrial Conglomerate</t>
+          <t>Money Center Bank</t>
         </is>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>37847</v>
+        <v>71355</v>
       </c>
       <c r="R24" s="3" t="inlineStr">
         <is>
@@ -2514,7 +2408,7 @@
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
@@ -2522,64 +2416,64 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>POD 6 Cyber Telco Retail M&amp;E</t>
+          <t>POD 4 Banking Payments Insurance</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Verizon Communications</t>
+          <t>Mastercard Incorporated</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>verizon.com</t>
+          <t>mastercard.com</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; +3 ML roles added</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J25" s="3" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>Principal Data Scientist</t>
+          <t>Principal AI Engineer</t>
         </is>
       </c>
       <c r="P25" s="3" t="inlineStr">
         <is>
-          <t>Telco</t>
+          <t>Payment Networks</t>
         </is>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>134788</v>
+        <v>28167</v>
       </c>
       <c r="R25" s="3" t="inlineStr">
         <is>
@@ -2595,7 +2489,7 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -2603,66 +2497,58 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>POD 3 Manufacturing &amp; Robotics</t>
+          <t>POD 4 Banking Payments Insurance</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Jacobs Solutions Inc.</t>
+          <t>Travelers Companies</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>jacobs.com</t>
+          <t>travelers.com</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G26" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +2 ML roles added</t>
+          <t>1 active ML roles</t>
         </is>
       </c>
       <c r="J26" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="N26" s="2" t="inlineStr"/>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>Senior AI/Data Platform Engineer (Snowflake, GenAI)</t>
+          <t>Senior Data &amp; AI Engineer</t>
         </is>
       </c>
       <c r="P26" s="3" t="inlineStr">
         <is>
-          <t>Engineering / Defense</t>
+          <t>P&amp;C Insurance</t>
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>16751</v>
+        <v>46421</v>
       </c>
       <c r="R26" s="3" t="inlineStr">
         <is>
@@ -2678,7 +2564,7 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
@@ -2701,33 +2587,29 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +2 ML roles added</t>
+          <t>Director+ hiring; GPU/inference signal</t>
         </is>
       </c>
       <c r="J27" s="3" t="n">
         <v>2</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="L27" s="2" t="inlineStr"/>
       <c r="M27" s="2" t="n">
         <v>1</v>
       </c>
@@ -2763,7 +2645,7 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -2771,68 +2653,58 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>POD 6 Cyber Telco Retail M&amp;E</t>
+          <t>POD 5 Consumer Internet Software Auto</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Paramount Global</t>
+          <t>Comcast Corporation</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>paramount.com</t>
+          <t>corporate.comcast.com</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Director+ hiring; GPU/inference signal; +2 ML roles added</t>
+          <t>1 active ML roles</t>
         </is>
       </c>
       <c r="J28" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>Principal Machine Learning Engineer, Presentation and Visual Optimization</t>
+          <t>Engineer 4 - Machine Learning</t>
         </is>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Cable / Media</t>
         </is>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>29206</v>
+        <v>123731</v>
       </c>
       <c r="R28" s="3" t="inlineStr">
         <is>
@@ -2848,7 +2720,7 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
@@ -2856,48 +2728,44 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>POD 4 Banking Payments Insurance</t>
+          <t>POD 5 Consumer Internet Software Auto</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>PayPal Holdings</t>
+          <t>Netflix Inc.</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>paypal.com</t>
+          <t>netflix.com</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +1 ML roles added</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J29" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="L29" s="2" t="inlineStr"/>
       <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr">
         <is>
@@ -2906,16 +2774,16 @@
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Sr Machine Learning Engineer — Agentic Systems</t>
+          <t>Data Scientist 5 - TV &amp; Interactive Discovery</t>
         </is>
       </c>
       <c r="P29" s="3" t="inlineStr">
         <is>
-          <t>Payments</t>
+          <t>Streaming</t>
         </is>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>31797</v>
+        <v>39001</v>
       </c>
       <c r="R29" s="3" t="inlineStr">
         <is>
@@ -2931,7 +2799,7 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -2939,62 +2807,62 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>POD 1 Capital Markets</t>
+          <t>POD 5 Consumer Internet Software Auto</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Intercontinental Exchange</t>
+          <t>Qualcomm Inc.</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>ice.com</t>
+          <t>qualcomm.com</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>+1 ML roles added</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J30" s="3" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
+        <v>29</v>
+      </c>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>2026 Intern-Machine Learning &amp;Multimedia Software Engineer</t>
         </is>
       </c>
       <c r="P30" s="3" t="inlineStr">
         <is>
-          <t>Exchanges</t>
+          <t>Semiconductors</t>
         </is>
       </c>
       <c r="Q30" s="2" t="n">
-        <v>9333</v>
+        <v>38962</v>
       </c>
       <c r="R30" s="3" t="inlineStr">
         <is>
@@ -3010,7 +2878,7 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
@@ -3018,62 +2886,62 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>POD 2 Healthcare &amp; Life Sciences</t>
+          <t>POD 5 Consumer Internet Software Auto</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Abbott Laboratories</t>
+          <t>Salesforce Inc.</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>abbott.com</t>
+          <t>salesforce.com</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>+1 ML roles added</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J31" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>Senior Clinical Research Scientist</t>
+          <t>Lead AI Engineer, Data Solutions</t>
         </is>
       </c>
       <c r="P31" s="3" t="inlineStr">
         <is>
-          <t>Medical Devices</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>41950</v>
+        <v>37895</v>
       </c>
       <c r="R31" s="3" t="inlineStr">
         <is>
@@ -3089,7 +2957,7 @@
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -3097,66 +2965,58 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>POD 3 Manufacturing &amp; Robotics</t>
+          <t>POD 5 Consumer Internet Software Auto</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Boeing Company</t>
+          <t>Stellantis N.V.</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>boeing.com</t>
+          <t>stellantis.com</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>GPU/inference signal; +1 ML roles added</t>
+          <t>1 active ML roles</t>
         </is>
       </c>
       <c r="J32" s="3" t="n">
         <v>1</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="L32" s="2" t="inlineStr"/>
       <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="3" t="inlineStr">
         <is>
-          <t>AI/ML Researcher (Multimodal)</t>
+          <t>Senior Data Scientist</t>
         </is>
       </c>
       <c r="P32" s="3" t="inlineStr">
         <is>
-          <t>Aerospace</t>
+          <t>Auto OEM</t>
         </is>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>77794</v>
+        <v>201202</v>
       </c>
       <c r="R32" s="3" t="inlineStr">
         <is>
@@ -3172,7 +3032,7 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
@@ -3180,62 +3040,62 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>POD 4 Banking Payments Insurance</t>
+          <t>POD 5 Consumer Internet Software Auto</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>AIG (American Intl. Group)</t>
+          <t>Tesla Inc.</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>aig.com</t>
+          <t>tesla.com</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G33" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>+1 ML roles added</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J33" s="3" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
+        <v>21</v>
+      </c>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>Ph.D. Research Data Scientist, GenAI</t>
+          <t>Site Reliability Engineer, HPC / AI Infrastructure</t>
         </is>
       </c>
       <c r="P33" s="3" t="inlineStr">
         <is>
-          <t>P&amp;C Insurance</t>
+          <t>EV / Auto</t>
         </is>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>46951</v>
+        <v>97690</v>
       </c>
       <c r="R33" s="3" t="inlineStr">
         <is>
@@ -3251,7 +3111,7 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -3259,62 +3119,64 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>POD 4 Banking Payments Insurance</t>
+          <t>POD 6 Cyber Telco Retail M&amp;E</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Travelers Companies</t>
+          <t>Paramount Global</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>travelers.com</t>
+          <t>paramount.com</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Director+ hiring; GPU/inference signal</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>+1 ML roles added</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K34" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>Senior Data &amp; AI Engineer</t>
+          <t>Principal Machine Learning Engineer, Presentation and Visual Optimization</t>
         </is>
       </c>
       <c r="P34" s="3" t="inlineStr">
         <is>
-          <t>P&amp;C Insurance</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>46421</v>
+        <v>29206</v>
       </c>
       <c r="R34" s="3" t="inlineStr">
         <is>
@@ -3330,7 +3192,7 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
@@ -3338,62 +3200,62 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>POD 5 Consumer Internet Software Auto</t>
+          <t>POD 6 Cyber Telco Retail M&amp;E</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Comcast Corporation</t>
+          <t>T-Mobile US Inc.</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>corporate.comcast.com</t>
+          <t>t-mobile.com</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>+1 ML roles added</t>
+          <t>GPU/inference signal</t>
         </is>
       </c>
       <c r="J35" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="2" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>Engineer 4 - Machine Learning</t>
+          <t>T Hub - AI Intern – LLM, Voice to Text &amp; Agentic Systems</t>
         </is>
       </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>Cable / Media</t>
+          <t>Telco</t>
         </is>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>123731</v>
+        <v>81400</v>
       </c>
       <c r="R35" s="3" t="inlineStr">
         <is>
@@ -3409,7 +3271,7 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Hot 🟩</t>
+          <t>Warm 🟨</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -3417,62 +3279,60 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>POD 5 Consumer Internet Software Auto</t>
+          <t>POD 6 Cyber Telco Retail M&amp;E</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Stellantis N.V.</t>
+          <t>Verizon Communications</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>stellantis.com</t>
+          <t>verizon.com</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Outbound Now — High ML Signal</t>
+          <t>Monitor — Trending Up</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Director+ hiring</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K36" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t>+1 ML roles added</t>
-        </is>
-      </c>
-      <c r="J36" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K36" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>Senior Data Scientist</t>
+          <t>Principal Data Scientist</t>
         </is>
       </c>
       <c r="P36" s="3" t="inlineStr">
         <is>
-          <t>Auto OEM</t>
+          <t>Telco</t>
         </is>
       </c>
       <c r="Q36" s="2" t="n">
-        <v>201202</v>
+        <v>134788</v>
       </c>
       <c r="R36" s="3" t="inlineStr">
         <is>

</xml_diff>